<commit_message>
Correcciones de la revisión: brigadistas solo bajo mina, ahorro por mejora, distancias y aclaraciones
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRADwuPWoSGgwKsv131MFz
</commit_message>
<xml_diff>
--- a/plan/Plan_100_dias_Servicio_Medico.xlsx
+++ b/plan/Plan_100_dias_Servicio_Medico.xlsx
@@ -158,7 +158,7 @@
     <t xml:space="preserve">Roster 8x6: la mitad del tiempo el equipo trabaja sin el Team Lead en sitio</t>
   </si>
   <si>
-    <t xml:space="preserve">Distancia: el hospital más cercano está a más de 2 horas por ruta</t>
+    <t xml:space="preserve">Distancia: el hospital más cercano está a dos o tres horas por ruta</t>
   </si>
   <si>
     <t xml:space="preserve">Logística: los insumos tardan entre 10 y 17 días en llegar</t>
@@ -404,7 +404,7 @@
     <t xml:space="preserve">Causas raíz priorizadas</t>
   </si>
   <si>
-    <t xml:space="preserve">Protocolo de derivación pre acordado con prestador y hospitales</t>
+    <t xml:space="preserve">Protocolo de derivación preacordado con prestador y hospitales</t>
   </si>
   <si>
     <t xml:space="preserve">Team Lead + Superintendente</t>
@@ -809,7 +809,7 @@
     <t xml:space="preserve">Definir</t>
   </si>
   <si>
-    <t xml:space="preserve">Según el modelo, en el escenario de referencia la ambulancia sale del sitio a las 2 h 19 min del aviso (mediana) y a las 2 h 53 min en el percentil 90. Ese tramo es casi la mitad (49%) del tiempo hasta el hospital más cercano, y es la parte que depende del servicio médico.</t>
+    <t xml:space="preserve">Según el modelo, en el escenario de referencia la ambulancia sale del sitio a las 2 h 19 min del aviso (mediana) y a las 2 h 53 min en el percentil 90. Ese tramo es casi la mitad (49%) del tiempo hasta el hospital más cercano, y es la parte que se resuelve dentro del sitio.</t>
   </si>
   <si>
     <t xml:space="preserve">Medir</t>
@@ -821,10 +821,10 @@
     <t xml:space="preserve">La coordinación de la derivación es la espera más larga: 41 min de mediana, y arranca recién cuando termina la estabilización. Son llamadas, búsqueda de cama y autorizaciones en serie.</t>
   </si>
   <si>
-    <t xml:space="preserve">Protocolo de derivación pre acordado (criterios escritos y un contacto único por hospital) y coordinación en paralelo a la estabilización. Ambulancia y chofer se preparan mientras tanto.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P90 del tiempo de salida en el tablero mensual. Resultado esperado según el modelo: 60 min menos en la mediana y 75 min menos en el P90.</t>
+    <t xml:space="preserve">Protocolo de derivación preacordado (criterios escritos y un contacto único por hospital) y coordinación en paralelo a la estabilización. Ambulancia y chofer se preparan mientras tanto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P90 del tiempo de salida en el tablero mensual. Resultado esperado según el modelo: 55 min menos en la mediana y 64 min menos en el P90 con esta mejora sola; 60 y 75 min sumando brigadistas bajo mina.</t>
   </si>
   <si>
     <t xml:space="preserve">Cero quiebres de stock crítico</t>
@@ -2445,11 +2445,11 @@
         <v>70</v>
       </c>
       <c r="F20" s="10" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="G20" s="11" t="n">
         <f aca="false">E20+F20-1</f>
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="H20" s="12"/>
       <c r="I20" s="12"/>

</xml_diff>

<commit_message>
Rediseño visual en toda la línea: página, PDF, carrusel y Excel
Tipografía Segoe UI con Selawik embebida, tarjetas redondeadas, degradados y paleta de BI.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRADwuPWoSGgwKsv131MFz
</commit_message>
<xml_diff>
--- a/plan/Plan_100_dias_Servicio_Medico.xlsx
+++ b/plan/Plan_100_dias_Servicio_Medico.xlsx
@@ -879,37 +879,36 @@
     <font>
       <b val="true"/>
       <sz val="14"/>
-      <color rgb="FF0B2545"/>
-      <name val="Arial"/>
+      <color rgb="FF0E1726"/>
+      <name val="Segoe UI"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
       <sz val="9"/>
-      <color rgb="FF5A6475"/>
-      <name val="Arial"/>
+      <color rgb="FF4B5563"/>
+      <name val="Segoe UI"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <name val="Arial"/>
+      <name val="Segoe UI"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
-      <name val="Arial"/>
+      <name val="Segoe UI"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FF0B2545"/>
-      <name val="Arial"/>
+      <color rgb="FF0E1726"/>
+      <name val="Segoe UI"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -917,36 +916,36 @@
       <b val="true"/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
+      <name val="Segoe UI"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FF5A6475"/>
-      <name val="Arial"/>
+      <name val="Segoe UI"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="7"/>
       <color rgb="FF5A6475"/>
-      <name val="Arial"/>
+      <name val="Segoe UI"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
-      <name val="Arial"/>
+      <name val="Segoe UI"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="12"/>
-      <color rgb="FF0B2545"/>
-      <name val="Arial"/>
+      <color rgb="FF0E1726"/>
+      <name val="Segoe UI"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -956,7 +955,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -965,20 +964,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0B2545"/>
-        <bgColor rgb="FF333333"/>
+        <fgColor rgb="FF0078D4"/>
+        <bgColor rgb="FF008080"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F5FA8"/>
-        <bgColor rgb="FF3366FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9731A"/>
-        <bgColor rgb="FFFF9900"/>
+        <fgColor rgb="FFE66C37"/>
+        <bgColor rgb="FFFF8080"/>
       </patternFill>
     </fill>
   </fills>
@@ -992,16 +985,16 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FFD5DBE5"/>
+        <color rgb="FFE1E1E1"/>
       </left>
       <right style="thin">
-        <color rgb="FFD5DBE5"/>
+        <color rgb="FFE1E1E1"/>
       </right>
       <top style="thin">
-        <color rgb="FFD5DBE5"/>
+        <color rgb="FFE1E1E1"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFD5DBE5"/>
+        <color rgb="FFE1E1E1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1116,11 +1109,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1137,28 +1130,28 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF1F5FA8"/>
+          <bgColor rgb="FF0078D4"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFF6D9BF"/>
+          <bgColor rgb="FFDCEEF8"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFF6D8D4"/>
+          <bgColor rgb="FFFDE7E9"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFBEBD3"/>
+          <bgColor rgb="FFFBE3D6"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1179,16 +1172,16 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFF6D8D4"/>
+      <rgbColor rgb="FFC0C0C0"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFBEBD3"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFFDE7E9"/>
+      <rgbColor rgb="FFDCEEF8"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF1F5FA8"/>
-      <rgbColor rgb="FFD5DBE5"/>
+      <rgbColor rgb="FF0078D4"/>
+      <rgbColor rgb="FFE1E1E1"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -1204,23 +1197,23 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFF6D9BF"/>
+      <rgbColor rgb="FFFBE3D6"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFD9731A"/>
+      <rgbColor rgb="FFE66C37"/>
       <rgbColor rgb="FF5A6475"/>
       <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF0B2545"/>
+      <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF0E1726"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="FF4B5563"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -1431,7 +1424,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
@@ -1506,7 +1499,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
         <v>16</v>
       </c>
@@ -1534,7 +1527,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="4" t="s">
         <v>22</v>
       </c>
@@ -1843,7 +1836,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
         <v>98</v>
       </c>
@@ -1882,7 +1875,7 @@
       <c r="U5" s="12"/>
       <c r="V5" s="12"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
         <v>101</v>
       </c>
@@ -2116,7 +2109,7 @@
       <c r="U11" s="12"/>
       <c r="V11" s="12"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
         <v>116</v>
       </c>
@@ -2467,7 +2460,7 @@
       <c r="U20" s="12"/>
       <c r="V20" s="12"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
         <v>140</v>
       </c>
@@ -2506,7 +2499,7 @@
       <c r="U21" s="12"/>
       <c r="V21" s="12"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
         <v>142</v>
       </c>
@@ -2545,7 +2538,7 @@
       <c r="U22" s="12"/>
       <c r="V22" s="12"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
         <v>144</v>
       </c>
@@ -2969,7 +2962,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
         <v>179</v>
       </c>
@@ -3315,7 +3308,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
         <v>219</v>
       </c>
@@ -3384,7 +3377,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
         <v>241</v>
       </c>
@@ -3407,7 +3400,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
         <v>246</v>
       </c>

</xml_diff>